<commit_message>
feat(cron): backfill history + fix footer
- history.json: add Oct 1-3 from git history (D-100: 814, D-99: 952, D-98: 1027)
- index.html: footer text corrected to "every hour" (cron is 17 * * * *)
- comparison.xlsx: regenerated with 4 JH 2027 data points
</commit_message>
<xml_diff>
--- a/comparison.xlsx
+++ b/comparison.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Pace Chart" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Pace Targets" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Live Breakdown" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="JH 2026 Raw" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pace Chart" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pace Targets" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Live Breakdown" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JH 2026 Raw" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -38,12 +38,12 @@
       <sz val="9"/>
     </font>
     <font>
-      <color rgb="00991B1B"/>
+      <b val="1"/>
+      <color rgb="00C2410C"/>
       <sz val="9"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="00C2410C"/>
+      <color rgb="00991B1B"/>
       <sz val="9"/>
     </font>
     <font>
@@ -240,14 +240,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -270,7 +270,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="20000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="20000">
               <a:solidFill>
                 <a:srgbClr val="1E3A5F"/>
               </a:solidFill>
@@ -280,7 +280,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -305,7 +305,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="25000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25000">
               <a:solidFill>
                 <a:srgbClr val="F97316"/>
               </a:solidFill>
@@ -315,7 +315,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -340,7 +340,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="14000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="14000">
               <a:solidFill>
                 <a:srgbClr val="DC2626"/>
               </a:solidFill>
@@ -350,7 +350,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -378,8 +378,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -405,8 +405,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -432,7 +432,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>5</col>
@@ -447,9 +447,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -782,7 +782,10 @@
       <c r="A2" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="C2" s="3" t="n">
+        <v>814</v>
+      </c>
+      <c r="D2" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -790,7 +793,10 @@
       <c r="A3" s="2" t="n">
         <v>99</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="C3" s="3" t="n">
+        <v>952</v>
+      </c>
+      <c r="D3" s="4" t="n">
         <v>97</v>
       </c>
     </row>
@@ -798,7 +804,10 @@
       <c r="A4" s="2" t="n">
         <v>98</v>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="C4" s="3" t="n">
+        <v>1027</v>
+      </c>
+      <c r="D4" s="4" t="n">
         <v>194</v>
       </c>
     </row>
@@ -806,10 +815,10 @@
       <c r="A5" s="2" t="n">
         <v>97</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="3" t="n">
         <v>1027</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D5" s="4" t="n">
         <v>290</v>
       </c>
     </row>
@@ -817,7 +826,7 @@
       <c r="A6" s="2" t="n">
         <v>96</v>
       </c>
-      <c r="D6" s="3" t="n">
+      <c r="D6" s="4" t="n">
         <v>387</v>
       </c>
     </row>
@@ -825,7 +834,7 @@
       <c r="A7" s="2" t="n">
         <v>95</v>
       </c>
-      <c r="D7" s="3" t="n">
+      <c r="D7" s="4" t="n">
         <v>484</v>
       </c>
     </row>
@@ -833,7 +842,7 @@
       <c r="A8" s="2" t="n">
         <v>94</v>
       </c>
-      <c r="D8" s="3" t="n">
+      <c r="D8" s="4" t="n">
         <v>581</v>
       </c>
     </row>
@@ -841,7 +850,7 @@
       <c r="A9" s="2" t="n">
         <v>93</v>
       </c>
-      <c r="D9" s="3" t="n">
+      <c r="D9" s="4" t="n">
         <v>677</v>
       </c>
     </row>
@@ -849,7 +858,7 @@
       <c r="A10" s="2" t="n">
         <v>92</v>
       </c>
-      <c r="D10" s="3" t="n">
+      <c r="D10" s="4" t="n">
         <v>774</v>
       </c>
     </row>
@@ -857,7 +866,7 @@
       <c r="A11" s="2" t="n">
         <v>91</v>
       </c>
-      <c r="D11" s="3" t="n">
+      <c r="D11" s="4" t="n">
         <v>871</v>
       </c>
     </row>
@@ -865,7 +874,7 @@
       <c r="A12" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="D12" s="3" t="n">
+      <c r="D12" s="4" t="n">
         <v>968</v>
       </c>
     </row>
@@ -873,7 +882,7 @@
       <c r="A13" s="2" t="n">
         <v>89</v>
       </c>
-      <c r="D13" s="3" t="n">
+      <c r="D13" s="4" t="n">
         <v>1065</v>
       </c>
     </row>
@@ -881,7 +890,7 @@
       <c r="A14" s="2" t="n">
         <v>88</v>
       </c>
-      <c r="D14" s="3" t="n">
+      <c r="D14" s="4" t="n">
         <v>1161</v>
       </c>
     </row>
@@ -889,7 +898,7 @@
       <c r="A15" s="2" t="n">
         <v>87</v>
       </c>
-      <c r="D15" s="3" t="n">
+      <c r="D15" s="4" t="n">
         <v>1258</v>
       </c>
     </row>
@@ -897,7 +906,7 @@
       <c r="A16" s="2" t="n">
         <v>86</v>
       </c>
-      <c r="D16" s="3" t="n">
+      <c r="D16" s="4" t="n">
         <v>1355</v>
       </c>
     </row>
@@ -905,7 +914,7 @@
       <c r="A17" s="2" t="n">
         <v>85</v>
       </c>
-      <c r="D17" s="3" t="n">
+      <c r="D17" s="4" t="n">
         <v>1452</v>
       </c>
     </row>
@@ -913,7 +922,7 @@
       <c r="A18" s="2" t="n">
         <v>84</v>
       </c>
-      <c r="D18" s="3" t="n">
+      <c r="D18" s="4" t="n">
         <v>1548</v>
       </c>
     </row>
@@ -921,7 +930,7 @@
       <c r="A19" s="2" t="n">
         <v>83</v>
       </c>
-      <c r="D19" s="3" t="n">
+      <c r="D19" s="4" t="n">
         <v>1645</v>
       </c>
     </row>
@@ -929,7 +938,7 @@
       <c r="A20" s="2" t="n">
         <v>82</v>
       </c>
-      <c r="D20" s="3" t="n">
+      <c r="D20" s="4" t="n">
         <v>1742</v>
       </c>
     </row>
@@ -937,7 +946,7 @@
       <c r="A21" s="2" t="n">
         <v>81</v>
       </c>
-      <c r="D21" s="3" t="n">
+      <c r="D21" s="4" t="n">
         <v>1839</v>
       </c>
     </row>
@@ -945,7 +954,7 @@
       <c r="A22" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="D22" s="3" t="n">
+      <c r="D22" s="4" t="n">
         <v>1935</v>
       </c>
     </row>
@@ -953,7 +962,7 @@
       <c r="A23" s="2" t="n">
         <v>79</v>
       </c>
-      <c r="D23" s="3" t="n">
+      <c r="D23" s="4" t="n">
         <v>2032</v>
       </c>
     </row>
@@ -961,7 +970,7 @@
       <c r="A24" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="D24" s="3" t="n">
+      <c r="D24" s="4" t="n">
         <v>2129</v>
       </c>
     </row>
@@ -969,7 +978,7 @@
       <c r="A25" s="2" t="n">
         <v>77</v>
       </c>
-      <c r="D25" s="3" t="n">
+      <c r="D25" s="4" t="n">
         <v>2226</v>
       </c>
     </row>
@@ -977,7 +986,7 @@
       <c r="A26" s="2" t="n">
         <v>76</v>
       </c>
-      <c r="D26" s="3" t="n">
+      <c r="D26" s="4" t="n">
         <v>2323</v>
       </c>
     </row>
@@ -985,7 +994,7 @@
       <c r="A27" s="2" t="n">
         <v>75</v>
       </c>
-      <c r="D27" s="3" t="n">
+      <c r="D27" s="4" t="n">
         <v>2419</v>
       </c>
     </row>
@@ -993,7 +1002,7 @@
       <c r="A28" s="2" t="n">
         <v>74</v>
       </c>
-      <c r="D28" s="3" t="n">
+      <c r="D28" s="4" t="n">
         <v>2516</v>
       </c>
     </row>
@@ -1001,7 +1010,7 @@
       <c r="A29" s="2" t="n">
         <v>73</v>
       </c>
-      <c r="D29" s="3" t="n">
+      <c r="D29" s="4" t="n">
         <v>2613</v>
       </c>
     </row>
@@ -1009,7 +1018,7 @@
       <c r="A30" s="2" t="n">
         <v>72</v>
       </c>
-      <c r="D30" s="3" t="n">
+      <c r="D30" s="4" t="n">
         <v>2710</v>
       </c>
     </row>
@@ -1017,7 +1026,7 @@
       <c r="A31" s="2" t="n">
         <v>71</v>
       </c>
-      <c r="D31" s="3" t="n">
+      <c r="D31" s="4" t="n">
         <v>2806</v>
       </c>
     </row>
@@ -1025,7 +1034,7 @@
       <c r="A32" s="2" t="n">
         <v>70</v>
       </c>
-      <c r="D32" s="3" t="n">
+      <c r="D32" s="4" t="n">
         <v>2903</v>
       </c>
     </row>
@@ -1033,7 +1042,7 @@
       <c r="A33" s="2" t="n">
         <v>69</v>
       </c>
-      <c r="D33" s="3" t="n">
+      <c r="D33" s="4" t="n">
         <v>3000</v>
       </c>
     </row>
@@ -1041,7 +1050,7 @@
       <c r="A34" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="D34" s="3" t="n">
+      <c r="D34" s="4" t="n">
         <v>3117</v>
       </c>
     </row>
@@ -1049,7 +1058,7 @@
       <c r="A35" s="2" t="n">
         <v>67</v>
       </c>
-      <c r="D35" s="3" t="n">
+      <c r="D35" s="4" t="n">
         <v>3233</v>
       </c>
     </row>
@@ -1057,7 +1066,7 @@
       <c r="A36" s="2" t="n">
         <v>66</v>
       </c>
-      <c r="D36" s="3" t="n">
+      <c r="D36" s="4" t="n">
         <v>3350</v>
       </c>
     </row>
@@ -1065,7 +1074,7 @@
       <c r="A37" s="2" t="n">
         <v>65</v>
       </c>
-      <c r="D37" s="3" t="n">
+      <c r="D37" s="4" t="n">
         <v>3467</v>
       </c>
     </row>
@@ -1073,7 +1082,7 @@
       <c r="A38" s="2" t="n">
         <v>64</v>
       </c>
-      <c r="D38" s="3" t="n">
+      <c r="D38" s="4" t="n">
         <v>3583</v>
       </c>
     </row>
@@ -1084,7 +1093,7 @@
       <c r="B39" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D39" s="3" t="n">
+      <c r="D39" s="4" t="n">
         <v>3700</v>
       </c>
     </row>
@@ -1095,7 +1104,7 @@
       <c r="B40" s="5" t="n">
         <v>1000</v>
       </c>
-      <c r="D40" s="3" t="n">
+      <c r="D40" s="4" t="n">
         <v>3817</v>
       </c>
     </row>
@@ -1103,7 +1112,7 @@
       <c r="A41" s="2" t="n">
         <v>61</v>
       </c>
-      <c r="D41" s="3" t="n">
+      <c r="D41" s="4" t="n">
         <v>3933</v>
       </c>
     </row>
@@ -1111,7 +1120,7 @@
       <c r="A42" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="D42" s="3" t="n">
+      <c r="D42" s="4" t="n">
         <v>4050</v>
       </c>
     </row>
@@ -1122,7 +1131,7 @@
       <c r="B43" s="5" t="n">
         <v>1200</v>
       </c>
-      <c r="D43" s="3" t="n">
+      <c r="D43" s="4" t="n">
         <v>4167</v>
       </c>
     </row>
@@ -1130,7 +1139,7 @@
       <c r="A44" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="D44" s="3" t="n">
+      <c r="D44" s="4" t="n">
         <v>4283</v>
       </c>
     </row>
@@ -1138,7 +1147,7 @@
       <c r="A45" s="2" t="n">
         <v>57</v>
       </c>
-      <c r="D45" s="3" t="n">
+      <c r="D45" s="4" t="n">
         <v>4400</v>
       </c>
     </row>
@@ -1146,7 +1155,7 @@
       <c r="A46" s="2" t="n">
         <v>56</v>
       </c>
-      <c r="D46" s="3" t="n">
+      <c r="D46" s="4" t="n">
         <v>4517</v>
       </c>
     </row>
@@ -1154,7 +1163,7 @@
       <c r="A47" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="D47" s="3" t="n">
+      <c r="D47" s="4" t="n">
         <v>4633</v>
       </c>
     </row>
@@ -1162,7 +1171,7 @@
       <c r="A48" s="2" t="n">
         <v>54</v>
       </c>
-      <c r="D48" s="3" t="n">
+      <c r="D48" s="4" t="n">
         <v>4750</v>
       </c>
     </row>
@@ -1170,7 +1179,7 @@
       <c r="A49" s="2" t="n">
         <v>53</v>
       </c>
-      <c r="D49" s="3" t="n">
+      <c r="D49" s="4" t="n">
         <v>4867</v>
       </c>
     </row>
@@ -1178,7 +1187,7 @@
       <c r="A50" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="D50" s="3" t="n">
+      <c r="D50" s="4" t="n">
         <v>4983</v>
       </c>
     </row>
@@ -1186,7 +1195,7 @@
       <c r="A51" s="2" t="n">
         <v>51</v>
       </c>
-      <c r="D51" s="3" t="n">
+      <c r="D51" s="4" t="n">
         <v>5100</v>
       </c>
     </row>
@@ -1194,7 +1203,7 @@
       <c r="A52" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="D52" s="3" t="n">
+      <c r="D52" s="4" t="n">
         <v>5217</v>
       </c>
     </row>
@@ -1205,7 +1214,7 @@
       <c r="B53" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="D53" s="3" t="n">
+      <c r="D53" s="4" t="n">
         <v>5333</v>
       </c>
     </row>
@@ -1213,7 +1222,7 @@
       <c r="A54" s="2" t="n">
         <v>48</v>
       </c>
-      <c r="D54" s="3" t="n">
+      <c r="D54" s="4" t="n">
         <v>5450</v>
       </c>
     </row>
@@ -1221,7 +1230,7 @@
       <c r="A55" s="2" t="n">
         <v>47</v>
       </c>
-      <c r="D55" s="3" t="n">
+      <c r="D55" s="4" t="n">
         <v>5567</v>
       </c>
     </row>
@@ -1229,7 +1238,7 @@
       <c r="A56" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="D56" s="3" t="n">
+      <c r="D56" s="4" t="n">
         <v>5683</v>
       </c>
     </row>
@@ -1237,7 +1246,7 @@
       <c r="A57" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="D57" s="3" t="n">
+      <c r="D57" s="4" t="n">
         <v>5800</v>
       </c>
     </row>
@@ -1245,7 +1254,7 @@
       <c r="A58" s="2" t="n">
         <v>44</v>
       </c>
-      <c r="D58" s="3" t="n">
+      <c r="D58" s="4" t="n">
         <v>5917</v>
       </c>
     </row>
@@ -1253,7 +1262,7 @@
       <c r="A59" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="D59" s="3" t="n">
+      <c r="D59" s="4" t="n">
         <v>6033</v>
       </c>
     </row>
@@ -1261,7 +1270,7 @@
       <c r="A60" s="2" t="n">
         <v>42</v>
       </c>
-      <c r="D60" s="3" t="n">
+      <c r="D60" s="4" t="n">
         <v>6150</v>
       </c>
     </row>
@@ -1269,7 +1278,7 @@
       <c r="A61" s="2" t="n">
         <v>41</v>
       </c>
-      <c r="D61" s="3" t="n">
+      <c r="D61" s="4" t="n">
         <v>6267</v>
       </c>
     </row>
@@ -1277,7 +1286,7 @@
       <c r="A62" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="D62" s="3" t="n">
+      <c r="D62" s="4" t="n">
         <v>6383</v>
       </c>
     </row>
@@ -1285,7 +1294,7 @@
       <c r="A63" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="D63" s="3" t="n">
+      <c r="D63" s="4" t="n">
         <v>6500</v>
       </c>
     </row>
@@ -1293,7 +1302,7 @@
       <c r="A64" s="2" t="n">
         <v>38</v>
       </c>
-      <c r="D64" s="3" t="n">
+      <c r="D64" s="4" t="n">
         <v>6677</v>
       </c>
     </row>
@@ -1301,7 +1310,7 @@
       <c r="A65" s="2" t="n">
         <v>37</v>
       </c>
-      <c r="D65" s="3" t="n">
+      <c r="D65" s="4" t="n">
         <v>6855</v>
       </c>
     </row>
@@ -1312,7 +1321,7 @@
       <c r="B66" s="5" t="n">
         <v>2000</v>
       </c>
-      <c r="D66" s="3" t="n">
+      <c r="D66" s="4" t="n">
         <v>7032</v>
       </c>
     </row>
@@ -1320,7 +1329,7 @@
       <c r="A67" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="D67" s="3" t="n">
+      <c r="D67" s="4" t="n">
         <v>7210</v>
       </c>
     </row>
@@ -1328,7 +1337,7 @@
       <c r="A68" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="D68" s="3" t="n">
+      <c r="D68" s="4" t="n">
         <v>7387</v>
       </c>
     </row>
@@ -1336,7 +1345,7 @@
       <c r="A69" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="D69" s="3" t="n">
+      <c r="D69" s="4" t="n">
         <v>7565</v>
       </c>
     </row>
@@ -1344,7 +1353,7 @@
       <c r="A70" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="D70" s="3" t="n">
+      <c r="D70" s="4" t="n">
         <v>7742</v>
       </c>
     </row>
@@ -1352,7 +1361,7 @@
       <c r="A71" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="D71" s="3" t="n">
+      <c r="D71" s="4" t="n">
         <v>7919</v>
       </c>
     </row>
@@ -1360,7 +1369,7 @@
       <c r="A72" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="D72" s="3" t="n">
+      <c r="D72" s="4" t="n">
         <v>8097</v>
       </c>
     </row>
@@ -1368,7 +1377,7 @@
       <c r="A73" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="D73" s="3" t="n">
+      <c r="D73" s="4" t="n">
         <v>8274</v>
       </c>
     </row>
@@ -1376,7 +1385,7 @@
       <c r="A74" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="D74" s="3" t="n">
+      <c r="D74" s="4" t="n">
         <v>8452</v>
       </c>
     </row>
@@ -1384,7 +1393,7 @@
       <c r="A75" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="D75" s="3" t="n">
+      <c r="D75" s="4" t="n">
         <v>8629</v>
       </c>
     </row>
@@ -1392,7 +1401,7 @@
       <c r="A76" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="D76" s="3" t="n">
+      <c r="D76" s="4" t="n">
         <v>8806</v>
       </c>
     </row>
@@ -1400,7 +1409,7 @@
       <c r="A77" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="D77" s="3" t="n">
+      <c r="D77" s="4" t="n">
         <v>8984</v>
       </c>
     </row>
@@ -1408,7 +1417,7 @@
       <c r="A78" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="D78" s="3" t="n">
+      <c r="D78" s="4" t="n">
         <v>9161</v>
       </c>
     </row>
@@ -1416,7 +1425,7 @@
       <c r="A79" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="D79" s="3" t="n">
+      <c r="D79" s="4" t="n">
         <v>9339</v>
       </c>
     </row>
@@ -1424,7 +1433,7 @@
       <c r="A80" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="D80" s="3" t="n">
+      <c r="D80" s="4" t="n">
         <v>9516</v>
       </c>
     </row>
@@ -1432,7 +1441,7 @@
       <c r="A81" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="D81" s="3" t="n">
+      <c r="D81" s="4" t="n">
         <v>9694</v>
       </c>
     </row>
@@ -1440,7 +1449,7 @@
       <c r="A82" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="D82" s="3" t="n">
+      <c r="D82" s="4" t="n">
         <v>9871</v>
       </c>
     </row>
@@ -1448,7 +1457,7 @@
       <c r="A83" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="D83" s="3" t="n">
+      <c r="D83" s="4" t="n">
         <v>10048</v>
       </c>
     </row>
@@ -1459,7 +1468,7 @@
       <c r="B84" s="5" t="n">
         <v>2358</v>
       </c>
-      <c r="D84" s="3" t="n">
+      <c r="D84" s="4" t="n">
         <v>10226</v>
       </c>
     </row>
@@ -1470,7 +1479,7 @@
       <c r="B85" s="5" t="n">
         <v>2412</v>
       </c>
-      <c r="D85" s="3" t="n">
+      <c r="D85" s="4" t="n">
         <v>10403</v>
       </c>
     </row>
@@ -1481,7 +1490,7 @@
       <c r="B86" s="5" t="n">
         <v>2465</v>
       </c>
-      <c r="D86" s="3" t="n">
+      <c r="D86" s="4" t="n">
         <v>10581</v>
       </c>
     </row>
@@ -1492,7 +1501,7 @@
       <c r="B87" s="5" t="n">
         <v>2689</v>
       </c>
-      <c r="D87" s="3" t="n">
+      <c r="D87" s="4" t="n">
         <v>10758</v>
       </c>
     </row>
@@ -1503,7 +1512,7 @@
       <c r="B88" s="5" t="n">
         <v>3201</v>
       </c>
-      <c r="D88" s="3" t="n">
+      <c r="D88" s="4" t="n">
         <v>10935</v>
       </c>
     </row>
@@ -1514,7 +1523,7 @@
       <c r="B89" s="5" t="n">
         <v>3447</v>
       </c>
-      <c r="D89" s="3" t="n">
+      <c r="D89" s="4" t="n">
         <v>11113</v>
       </c>
     </row>
@@ -1525,7 +1534,7 @@
       <c r="B90" s="5" t="n">
         <v>3675</v>
       </c>
-      <c r="D90" s="3" t="n">
+      <c r="D90" s="4" t="n">
         <v>11290</v>
       </c>
     </row>
@@ -1536,7 +1545,7 @@
       <c r="B91" s="5" t="n">
         <v>3884</v>
       </c>
-      <c r="D91" s="3" t="n">
+      <c r="D91" s="4" t="n">
         <v>11468</v>
       </c>
     </row>
@@ -1547,7 +1556,7 @@
       <c r="B92" s="5" t="n">
         <v>4054</v>
       </c>
-      <c r="D92" s="3" t="n">
+      <c r="D92" s="4" t="n">
         <v>11645</v>
       </c>
     </row>
@@ -1558,7 +1567,7 @@
       <c r="B93" s="5" t="n">
         <v>4309</v>
       </c>
-      <c r="D93" s="3" t="n">
+      <c r="D93" s="4" t="n">
         <v>11823</v>
       </c>
     </row>
@@ -1569,7 +1578,7 @@
       <c r="B94" s="5" t="n">
         <v>4620</v>
       </c>
-      <c r="D94" s="3" t="n">
+      <c r="D94" s="4" t="n">
         <v>12000</v>
       </c>
     </row>
@@ -1580,7 +1589,7 @@
       <c r="B95" s="5" t="n">
         <v>5002</v>
       </c>
-      <c r="D95" s="3" t="n">
+      <c r="D95" s="4" t="n">
         <v>12750</v>
       </c>
     </row>
@@ -1591,7 +1600,7 @@
       <c r="B96" s="5" t="n">
         <v>5300</v>
       </c>
-      <c r="D96" s="3" t="n">
+      <c r="D96" s="4" t="n">
         <v>13500</v>
       </c>
     </row>
@@ -1602,7 +1611,7 @@
       <c r="B97" s="5" t="n">
         <v>5663</v>
       </c>
-      <c r="D97" s="3" t="n">
+      <c r="D97" s="4" t="n">
         <v>14250</v>
       </c>
     </row>
@@ -1613,7 +1622,7 @@
       <c r="B98" s="5" t="n">
         <v>6277</v>
       </c>
-      <c r="D98" s="3" t="n">
+      <c r="D98" s="4" t="n">
         <v>15000</v>
       </c>
     </row>
@@ -1624,7 +1633,7 @@
       <c r="B99" s="5" t="n">
         <v>6805</v>
       </c>
-      <c r="D99" s="3" t="n">
+      <c r="D99" s="4" t="n">
         <v>15750</v>
       </c>
     </row>
@@ -1635,7 +1644,7 @@
       <c r="B100" s="5" t="n">
         <v>7309</v>
       </c>
-      <c r="D100" s="3" t="n">
+      <c r="D100" s="4" t="n">
         <v>16500</v>
       </c>
     </row>
@@ -1646,7 +1655,7 @@
       <c r="B101" s="5" t="n">
         <v>8059</v>
       </c>
-      <c r="D101" s="3" t="n">
+      <c r="D101" s="4" t="n">
         <v>17250</v>
       </c>
     </row>
@@ -1657,7 +1666,7 @@
       <c r="B102" s="5" t="n">
         <v>9850</v>
       </c>
-      <c r="D102" s="3" t="n">
+      <c r="D102" s="4" t="n">
         <v>18000</v>
       </c>
     </row>
@@ -1668,7 +1677,7 @@
       <c r="B103" s="5" t="n">
         <v>11500</v>
       </c>
-      <c r="D103" s="3" t="n">
+      <c r="D103" s="4" t="n">
         <v>18000</v>
       </c>
     </row>
@@ -1679,7 +1688,7 @@
       <c r="B104" s="5" t="n">
         <v>12100</v>
       </c>
-      <c r="D104" s="3" t="n">
+      <c r="D104" s="4" t="n">
         <v>18000</v>
       </c>
     </row>

</xml_diff>